<commit_message>
Shop: product shots without the apology written on them
The pictures were carrying a RENDERING tag on the card and PLACEHOLDER
burnt into the corner of the image. That was me hedging about art I had
drawn rather than photographed, twice over, on every card. It made a
working shop look unfinished, which is a worse problem than the one it
was warning about.

So: watermark gone, tags off, and the renders redone to look like product
shots -- a lit sweep behind the part, a fainter reflection under it, a
tighter shadow.

The mechanism stays. The spreadsheet's last column still turns the tag on
per product if a picture ever needs flagging, and the CSS rule stays with
it. Dropping a real photo over any file in images/shop/ at 900x630 still
needs no edit to the page.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MP3asA2N7V14sqBEfc9nwz
</commit_message>
<xml_diff>
--- a/shop-prices.xlsx
+++ b/shop-prices.xlsx
@@ -684,7 +684,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>

</xml_diff>